<commit_message>
Automatická aktualizace překladové databáze z webové aplikace
</commit_message>
<xml_diff>
--- a/translate-PL.xlsx
+++ b/translate-PL.xlsx
@@ -9661,7 +9661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9697,6 +9697,18 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>VMK11B - 120x200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dřevěná postel 80x200 masiv borovice - VMK10F</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VMK11B - 80x200</t>
         </is>
       </c>
     </row>

</xml_diff>